<commit_message>
make some updates for the optimizations
</commit_message>
<xml_diff>
--- a/public/assets/vendor_products_demo.xlsx
+++ b/public/assets/vendor_products_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\eramo-multi-vendor\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E120C5B-501D-469D-A575-998D800106C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E13B96-6BF2-43D8-B5AC-8E833DFFAC01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,15 +17,13 @@
     <sheet name="images" sheetId="2" r:id="rId2"/>
     <sheet name="variants" sheetId="3" r:id="rId3"/>
     <sheet name="variant_stock" sheetId="4" r:id="rId4"/>
-    <sheet name="occasions" sheetId="5" r:id="rId5"/>
-    <sheet name="occasion_products" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="179021" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="75">
   <si>
     <t>id</t>
   </si>
@@ -168,63 +166,6 @@
     <t>region_id</t>
   </si>
   <si>
-    <t>name_en</t>
-  </si>
-  <si>
-    <t>name_ar</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>end_date</t>
-  </si>
-  <si>
-    <t>Ramadan Offers</t>
-  </si>
-  <si>
-    <t>عروض رمضان</t>
-  </si>
-  <si>
-    <t>Best Ramadan Deals</t>
-  </si>
-  <si>
-    <t>أفضل عروض رمضان</t>
-  </si>
-  <si>
-    <t>Limited time</t>
-  </si>
-  <si>
-    <t>لفترة محدودة</t>
-  </si>
-  <si>
-    <t>Eid Offers</t>
-  </si>
-  <si>
-    <t>عروض العيد</t>
-  </si>
-  <si>
-    <t>Eid Specials</t>
-  </si>
-  <si>
-    <t>خصومات العيد</t>
-  </si>
-  <si>
-    <t>While stock lasts</t>
-  </si>
-  <si>
-    <t>حتى نفاذ الكمية</t>
-  </si>
-  <si>
-    <t>occasion_id</t>
-  </si>
-  <si>
-    <t>special_price</t>
-  </si>
-  <si>
-    <t>position</t>
-  </si>
-  <si>
     <t>features_en</t>
   </si>
   <si>
@@ -307,36 +248,12 @@
   </si>
   <si>
     <t>variant_sku</t>
-  </si>
-  <si>
-    <t>sub_title_en</t>
-  </si>
-  <si>
-    <t>sub_title_ar</t>
-  </si>
-  <si>
-    <t>meta title en</t>
-  </si>
-  <si>
-    <t>ميتا تيتل عربي</t>
-  </si>
-  <si>
-    <t>first-second-third</t>
-  </si>
-  <si>
-    <t>اول-ثانى-ثالث</t>
-  </si>
-  <si>
-    <t>is_active</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -378,13 +295,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -712,7 +626,7 @@
         <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -736,28 +650,28 @@
         <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="U1" t="s">
         <v>7</v>
@@ -766,16 +680,16 @@
         <v>8</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="AA1" t="s">
         <v>13</v>
@@ -828,40 +742,40 @@
         <v>29</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="U2" t="s">
         <v>25</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="Y2" t="s">
         <v>26</v>
@@ -920,40 +834,40 @@
         <v>40</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="U3" t="s">
         <v>36</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="Y3" t="s">
         <v>37</v>
@@ -998,7 +912,7 @@
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1006,7 +920,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>19</v>
@@ -1017,7 +931,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>30</v>
@@ -1048,7 +962,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>42</v>
@@ -1111,7 +1025,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>46</v>
@@ -1151,256 +1065,6 @@
       </c>
       <c r="C4">
         <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:S3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="13" width="20.6640625" customWidth="1"/>
-    <col min="14" max="15" width="20.6640625" style="4" customWidth="1"/>
-    <col min="16" max="16" width="38" style="4" customWidth="1"/>
-    <col min="17" max="17" width="24.5546875" customWidth="1"/>
-    <col min="18" max="24" width="20.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="N2" s="3">
-        <v>45785</v>
-      </c>
-      <c r="O2" s="3">
-        <v>45785</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="N3" s="3">
-        <v>45785</v>
-      </c>
-      <c r="O3" s="3">
-        <v>45785</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="P2" r:id="rId1" xr:uid="{0564E689-CD70-4D38-A606-A8CDA61D4258}"/>
-    <hyperlink ref="P3" r:id="rId2" xr:uid="{F599F08E-1F0B-4AE5-8F82-29182A0B2314}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="5" width="43.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>150</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>160</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>